<commit_message>
Update Banxico_Minutes_Analysis.xlsx - 2026-07-11
</commit_message>
<xml_diff>
--- a/Banxico_Minutes_Analysis.xlsx
+++ b/Banxico_Minutes_Analysis.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7930,6 +7930,66 @@
       <c r="L125" t="inlineStr">
         <is>
           <t>The decision to hold rates suggests stability in the near term, but ongoing geopolitical tensions could lead to volatility in yields and FX markets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Hold the policy rate steady.</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>{"cut_25": 0, "hold": 5, "raise_25": 0}</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>The global economy is expanding at a similar pace to the previous quarter, with emerging markets moderating and advanced economies showing a heterogeneous recovery. The US economy is growing faster than most advanced economies, driven by private consumption and non-residential investment in technology sectors.</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Global inflation continues to rise, mainly due to energy prices. Headline inflation in the US increased from 3.3% to 4.2%, with core inflation rising from 2.6% to 2.9%. Inflation expectations remain anchored, but there are concerns about potential future pressures from supply chain disruptions and high fertilizer prices.</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>The US labor market is stable with job creation and a steady unemployment rate. Risks to the labor market have decreased, but recent dynamics are driven by sectors like leisure and hospitality.</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>There were no dissents in the decision to hold the policy rate. The committee is unified in its cautious approach, focusing on inflation and external risks.</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>The committee emphasizes the commitment to price stability. Future policy will be data-dependent, with a focus on inflation dynamics and external risks.</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>The decision to hold rates suggests stability in the short term, with markets likely to focus on external developments and inflation data for future rate expectations.</t>
         </is>
       </c>
     </row>
@@ -7944,7 +8004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D125"/>
+  <dimension ref="A1:D126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10446,6 +10506,26 @@
       <c r="D125" t="inlineStr">
         <is>
           <t>The policy decision was to hold the interest rate steady.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>0</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Hold the policy rate steady.</t>
         </is>
       </c>
     </row>
@@ -10460,7 +10540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C540"/>
+  <dimension ref="A1:C544"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19640,6 +19720,74 @@
       <c r="C540" t="inlineStr">
         <is>
           <t>Labor markets show signs of cooling, reducing inflationary pressures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Global inflation continues to rise due to energy prices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Inflation expectations for the end of 2026 have been revised upwards in various countries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Recent negotiations have eased concerns about energy supply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>The US labor market risks have decreased, with stable job creation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Banxico_Minutes_Analysis.xlsx - 2026-08-22
</commit_message>
<xml_diff>
--- a/Banxico_Minutes_Analysis.xlsx
+++ b/Banxico_Minutes_Analysis.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7810,186 +7810,6 @@
       <c r="L123" t="inlineStr">
         <is>
           <t>The decision to hold rates suggests stability in the near term, but markets may anticipate future cuts if inflation continues to moderate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>2026-04-09</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>The policy decision was to hold the interest rate steady.</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="E124" t="n">
-        <v>0</v>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>{"cut_25": 0, "hold": 5}</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>The committee noted a slowdown in economic activity, with GDP growth decelerating in 2025 and showing signs of reactivation in late 2025, but with a contraction in early 2026.</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>Inflation remains a concern with global uncertainties adding risks. Headline inflation is expected to face upward pressure due to geopolitical tensions, although some economies are seeing inflation move towards central bank targets.</t>
-        </is>
-      </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>The labor market in the US shows signs of moderation with a slight increase in unemployment, indicating a cooling labor market.</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>There was a consensus to hold rates, with no significant dissent. The focus was on monitoring geopolitical risks and their economic impacts.</t>
-        </is>
-      </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>The committee remains cautious, highlighting the need to monitor geopolitical developments and their impact on inflation and growth. Future policy moves will depend on the evolution of these risks.</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t>The decision to hold rates suggests a cautious approach, likely leading to stable short-term yields. However, geopolitical risks could lead to volatility in FX markets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>The policy decision was to hold the interest rate steady.</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="E125" t="n">
-        <v>0</v>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>{"hold": 5}</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>The committee noted a contraction in Mexico's economic activity in Q1 2026, reversing gains from late 2025. Global growth is expected to expand at a slower pace due to geopolitical tensions.</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>Global inflation has risen due to energy prices, but medium- and long-term expectations remain anchored. In Mexico, inflationary pressures are noted but are expected to be temporary.</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>Labor markets in advanced economies show signs of cooling, with limited inflationary pressure from employment. In the US, labor participation and demand have moderated.</t>
-        </is>
-      </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t>There was a consensus to hold rates, with no dissenting votes. The committee expressed a range of views on the potential duration and impact of geopolitical tensions.</t>
-        </is>
-      </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>The committee remains cautious, prepared to adjust policy if necessary, depending on geopolitical developments and their impact on inflation and growth.</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t>The decision to hold rates suggests stability in the near term, but ongoing geopolitical tensions could lead to volatility in yields and FX markets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>2026-07-09</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Hold the policy rate steady.</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="E126" t="n">
-        <v>0</v>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>{"cut_25": 0, "hold": 5, "raise_25": 0}</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>The global economy is expanding at a similar pace to the previous quarter, with emerging markets moderating and advanced economies showing a heterogeneous recovery. The US economy is growing faster than most advanced economies, driven by private consumption and non-residential investment in technology sectors.</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>Global inflation continues to rise, mainly due to energy prices. Headline inflation in the US increased from 3.3% to 4.2%, with core inflation rising from 2.6% to 2.9%. Inflation expectations remain anchored, but there are concerns about potential future pressures from supply chain disruptions and high fertilizer prices.</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>The US labor market is stable with job creation and a steady unemployment rate. Risks to the labor market have decreased, but recent dynamics are driven by sectors like leisure and hospitality.</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t>There were no dissents in the decision to hold the policy rate. The committee is unified in its cautious approach, focusing on inflation and external risks.</t>
-        </is>
-      </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>The committee emphasizes the commitment to price stability. Future policy will be data-dependent, with a focus on inflation dynamics and external risks.</t>
-        </is>
-      </c>
-      <c r="L126" t="inlineStr">
-        <is>
-          <t>The decision to hold rates suggests stability in the short term, with markets likely to focus on external developments and inflation data for future rate expectations.</t>
         </is>
       </c>
     </row>
@@ -8004,7 +7824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10466,66 +10286,6 @@
       <c r="D123" t="inlineStr">
         <is>
           <t>Hold</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="B124" t="n">
-        <v>0</v>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>The policy decision was to hold the interest rate steady.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="B125" t="n">
-        <v>0</v>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>The policy decision was to hold the interest rate steady.</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="B126" t="n">
-        <v>0</v>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>Hold the policy rate steady.</t>
         </is>
       </c>
     </row>
@@ -10540,7 +10300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C544"/>
+  <dimension ref="A1:C532"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19584,210 +19344,6 @@
       <c r="C532" t="inlineStr">
         <is>
           <t>Risks from geopolitical tensions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="533">
-      <c r="A533" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="B533" t="inlineStr">
-        <is>
-          <t>hawkish</t>
-        </is>
-      </c>
-      <c r="C533" t="inlineStr">
-        <is>
-          <t>Geopolitical tensions in the Middle East have increased oil prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="534">
-      <c r="A534" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="B534" t="inlineStr">
-        <is>
-          <t>hawkish</t>
-        </is>
-      </c>
-      <c r="C534" t="inlineStr">
-        <is>
-          <t>Global inflation risks are heightened due to uncertainty.</t>
-        </is>
-      </c>
-    </row>
-    <row r="535">
-      <c r="A535" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="B535" t="inlineStr">
-        <is>
-          <t>dovish</t>
-        </is>
-      </c>
-      <c r="C535" t="inlineStr">
-        <is>
-          <t>The US labor market shows signs of cooling, with increased unemployment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="536">
-      <c r="A536" t="inlineStr">
-        <is>
-          <t>2026-03-26</t>
-        </is>
-      </c>
-      <c r="B536" t="inlineStr">
-        <is>
-          <t>dovish</t>
-        </is>
-      </c>
-      <c r="C536" t="inlineStr">
-        <is>
-          <t>Some central banks maintained their rates unchanged, reflecting caution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="537">
-      <c r="A537" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="B537" t="inlineStr">
-        <is>
-          <t>hawkish</t>
-        </is>
-      </c>
-      <c r="C537" t="inlineStr">
-        <is>
-          <t>Global inflation has increased due to energy prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="538">
-      <c r="A538" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="B538" t="inlineStr">
-        <is>
-          <t>hawkish</t>
-        </is>
-      </c>
-      <c r="C538" t="inlineStr">
-        <is>
-          <t>Geopolitical tensions could lead to persistent inflationary pressures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="539">
-      <c r="A539" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="B539" t="inlineStr">
-        <is>
-          <t>dovish</t>
-        </is>
-      </c>
-      <c r="C539" t="inlineStr">
-        <is>
-          <t>Medium- and long-term inflation expectations remain anchored.</t>
-        </is>
-      </c>
-    </row>
-    <row r="540">
-      <c r="A540" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="B540" t="inlineStr">
-        <is>
-          <t>dovish</t>
-        </is>
-      </c>
-      <c r="C540" t="inlineStr">
-        <is>
-          <t>Labor markets show signs of cooling, reducing inflationary pressures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="541">
-      <c r="A541" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="B541" t="inlineStr">
-        <is>
-          <t>hawkish</t>
-        </is>
-      </c>
-      <c r="C541" t="inlineStr">
-        <is>
-          <t>Global inflation continues to rise due to energy prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="542">
-      <c r="A542" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="B542" t="inlineStr">
-        <is>
-          <t>hawkish</t>
-        </is>
-      </c>
-      <c r="C542" t="inlineStr">
-        <is>
-          <t>Inflation expectations for the end of 2026 have been revised upwards in various countries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="543">
-      <c r="A543" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="B543" t="inlineStr">
-        <is>
-          <t>dovish</t>
-        </is>
-      </c>
-      <c r="C543" t="inlineStr">
-        <is>
-          <t>Recent negotiations have eased concerns about energy supply.</t>
-        </is>
-      </c>
-    </row>
-    <row r="544">
-      <c r="A544" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="B544" t="inlineStr">
-        <is>
-          <t>dovish</t>
-        </is>
-      </c>
-      <c r="C544" t="inlineStr">
-        <is>
-          <t>The US labor market risks have decreased, with stable job creation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Banxico_Minutes_Analysis.xlsx - 2026-08-23
</commit_message>
<xml_diff>
--- a/Banxico_Minutes_Analysis.xlsx
+++ b/Banxico_Minutes_Analysis.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7810,6 +7810,246 @@
       <c r="L123" t="inlineStr">
         <is>
           <t>The decision to hold rates suggests stability in the near term, but markets may anticipate future cuts if inflation continues to moderate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>The policy decision was to hold the interest rate steady.</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>0</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>{"cut_25": 0, "hold": 5}</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>The committee noted a slowdown in economic activity, with GDP growth decelerating in 2025 and showing signs of reactivation in late 2025, but with a contraction in early 2026.</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Inflation remains a concern with global uncertainties adding risks. Headline inflation is expected to face upward pressure due to geopolitical tensions, although some economies are seeing inflation move towards central bank targets.</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>The labor market in the US shows signs of moderation with a slight increase in unemployment, indicating a cooling labor market.</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>There was a consensus to hold rates, with no significant dissent. The focus was on monitoring geopolitical risks and their economic impacts.</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>The committee remains cautious, highlighting the need to monitor geopolitical developments and their impact on inflation and growth. Future policy moves will depend on the evolution of these risks.</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>The decision to hold rates suggests a cautious approach, likely leading to stable short-term yields. However, geopolitical risks could lead to volatility in FX markets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>The policy decision was to hold the interest rate steady.</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>{"hold": 5}</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>The committee noted a contraction in Mexico's economic activity in Q1 2026, reversing gains from late 2025. Global growth is expected to expand at a slower pace due to geopolitical tensions.</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Global inflation has risen due to energy prices, but medium- and long-term expectations remain anchored. In Mexico, inflationary pressures are noted but are expected to be temporary.</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Labor markets in advanced economies show signs of cooling, with limited inflationary pressure from employment. In the US, labor participation and demand have moderated.</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>There was a consensus to hold rates, with no dissenting votes. The committee expressed a range of views on the potential duration and impact of geopolitical tensions.</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>The committee remains cautious, prepared to adjust policy if necessary, depending on geopolitical developments and their impact on inflation and growth.</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>The decision to hold rates suggests stability in the near term, but ongoing geopolitical tensions could lead to volatility in yields and FX markets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Hold the policy rate steady.</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>{"cut_25": 0, "hold": 5, "raise_25": 0}</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>The global economy is expanding at a similar pace to the previous quarter, with emerging markets moderating and advanced economies showing a heterogeneous recovery. The US economy is growing faster than most advanced economies, driven by private consumption and non-residential investment in technology sectors.</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Global inflation continues to rise, mainly due to energy prices. Headline inflation in the US increased from 3.3% to 4.2%, with core inflation rising from 2.6% to 2.9%. Inflation expectations remain anchored, but there are concerns about potential future pressures from supply chain disruptions and high fertilizer prices.</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>The US labor market is stable with job creation and a steady unemployment rate. Risks to the labor market have decreased, but recent dynamics are driven by sectors like leisure and hospitality.</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>There were no dissents in the decision to hold the policy rate. The committee is unified in its cautious approach, focusing on inflation and external risks.</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>The committee emphasizes the commitment to price stability. Future policy will be data-dependent, with a focus on inflation dynamics and external risks.</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>The decision to hold rates suggests stability in the short term, with markets likely to focus on external developments and inflation data for future rate expectations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Hold the policy rate steady.</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>{"hold": 5, "raise_25": 3}</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>The Mexican economy showed expansion in Q2 2026, reversing the previous quarter's contraction, with positive contributions from all major sectors.</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Global inflation pressures persist due to geopolitical conflicts, with energy prices remaining volatile. Domestic inflation is influenced by external factors, but core inflation shows signs of moderation.</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>The labor market in the US remains stable with a decrease in downside risks, supporting domestic demand.</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>There was a split in views regarding the rate decision, with some members advocating for a rate increase due to persistent inflation risks, while others preferred to hold rates steady amid global uncertainties.</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>The committee remains data-dependent, monitoring global developments and inflationary pressures closely, with no clear signal on the next move.</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>The decision to hold rates suggests a cautious approach, likely keeping the yield curve stable in the short term, but with potential upward pressure if inflation risks materialize.</t>
         </is>
       </c>
     </row>
@@ -7824,7 +8064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D123"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10286,6 +10526,86 @@
       <c r="D123" t="inlineStr">
         <is>
           <t>Hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>0</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>The policy decision was to hold the interest rate steady.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>0</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>The policy decision was to hold the interest rate steady.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>0</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Hold the policy rate steady.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>0</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Hold the policy rate steady.</t>
         </is>
       </c>
     </row>
@@ -10300,7 +10620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C532"/>
+  <dimension ref="A1:C548"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19344,6 +19664,278 @@
       <c r="C532" t="inlineStr">
         <is>
           <t>Risks from geopolitical tensions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Geopolitical tensions in the Middle East have increased oil prices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Global inflation risks are heightened due to uncertainty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>The US labor market shows signs of cooling, with increased unemployment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Some central banks maintained their rates unchanged, reflecting caution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Global inflation has increased due to energy prices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Geopolitical tensions could lead to persistent inflationary pressures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Medium- and long-term inflation expectations remain anchored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Labor markets show signs of cooling, reducing inflationary pressures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Global inflation continues to rise due to energy prices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Inflation expectations for the end of 2026 have been revised upwards in various countries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Recent negotiations have eased concerns about energy supply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>The US labor market risks have decreased, with stable job creation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Persistent global inflation risks due to geopolitical tensions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>hawkish</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Expectation of a potential rate increase by the Federal Reserve in late 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Core inflation in advanced economies shows signs of moderation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>dovish</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>The Mexican economy rebounded in Q2 2026, reducing immediate concerns.</t>
         </is>
       </c>
     </row>

</xml_diff>